<commit_message>
Resources workbook: count all booklets with a known page count in the paper totals
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015a1BVf44TxxDmPSgmtdhzK
</commit_message>
<xml_diff>
--- a/00_Requisition/Resources_Weeks_1_to_10_Y7_Y8.xlsx
+++ b/00_Requisition/Resources_Weeks_1_to_10_Y7_Y8.xlsx
@@ -297,22 +297,22 @@
     <t xml:space="preserve">booklets; A5 saddle-stitched, 24 pages (6 A4 sheets folded and stapled twice), 90 gsm (1 per student plus 4 spares)</t>
   </si>
   <si>
+    <t xml:space="preserve">Handed out with the logbook; name and class on the cover; open in every lesson but closed and put away during the skills check; 4 spares kept with the logbook spares.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, see note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goes to 28 pages (7 sheets each) if the entries need more room; the requisition row gives neither the page count nor 90 gsm. The dictionary file says hand out in Week 1 with the logbook; the language pack allows Week 1 or the next lesson.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scientist's Logbook, Year 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">booklets; A5, one page per week (page count not stated)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Booklet (reprographics)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Handed out with the logbook; name and class on the cover; open in every lesson but closed and put away during the skills check; 4 spares kept with the logbook spares.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes, see note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goes to 28 pages (7 sheets each) if the entries need more room; the requisition row gives neither the page count nor 90 gsm. The dictionary file says hand out in Week 1 with the logbook; the language pack allows Week 1 or the next lesson.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scientist's Logbook, Year 7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">booklets; A5, one page per week (page count not stated)</t>
   </si>
   <si>
     <t xml:space="preserve">First page written in Think and Reflect ('What I did', and 'New words' if time); collected into the class box at the end of every lesson.</t>
@@ -9797,7 +9797,7 @@
       </c>
       <c r="O5" s="9" t="n">
         <f aca="false">SUMIFS($L$9:$L$721,$J$9:$J$721,M5)</f>
-        <v>196</v>
+        <v>364</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10393,7 +10393,7 @@
         <v>28</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="K19" s="11" t="n">
         <v>6</v>
@@ -10403,15 +10403,15 @@
         <v>168</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N19" s="11"/>
       <c r="O19" s="12"/>
       <c r="P19" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q19" s="13" t="s">
         <v>91</v>
-      </c>
-      <c r="Q19" s="13" t="s">
-        <v>92</v>
       </c>
       <c r="R19" s="11"/>
     </row>
@@ -10426,13 +10426,13 @@
         <v>40</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E20" s="11" t="n">
         <v>24</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G20" s="11" t="s">
         <v>43</v>
@@ -10443,7 +10443,7 @@
         <v>24</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="K20" s="11"/>
       <c r="L20" s="11" t="str">
@@ -10506,7 +10506,7 @@
       <c r="N21" s="11"/>
       <c r="O21" s="12"/>
       <c r="P21" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q21" s="13" t="s">
         <v>101</v>
@@ -10554,7 +10554,7 @@
       </c>
       <c r="O22" s="12"/>
       <c r="P22" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>106</v>
@@ -10780,7 +10780,7 @@
       <c r="N27" s="11"/>
       <c r="O27" s="12"/>
       <c r="P27" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q27" s="13" t="s">
         <v>123</v>
@@ -11008,7 +11008,7 @@
       <c r="N32" s="11"/>
       <c r="O32" s="12"/>
       <c r="P32" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q32" s="13" t="s">
         <v>148</v>
@@ -11981,7 +11981,7 @@
         <v>24</v>
       </c>
       <c r="J52" s="12" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="K52" s="11"/>
       <c r="L52" s="11" t="str">
@@ -12464,7 +12464,7 @@
       <c r="N62" s="11"/>
       <c r="O62" s="12"/>
       <c r="P62" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q62" s="13" t="s">
         <v>252</v>
@@ -12508,7 +12508,7 @@
       <c r="N63" s="11"/>
       <c r="O63" s="12"/>
       <c r="P63" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q63" s="13" t="s">
         <v>256</v>
@@ -13282,7 +13282,7 @@
       <c r="N80" s="11"/>
       <c r="O80" s="12"/>
       <c r="P80" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q80" s="13" t="s">
         <v>316</v>
@@ -13466,7 +13466,7 @@
       </c>
       <c r="O84" s="12"/>
       <c r="P84" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q84" s="13" t="s">
         <v>329</v>
@@ -13996,7 +13996,7 @@
         <v>365</v>
       </c>
       <c r="P95" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q95" s="13" t="s">
         <v>366</v>
@@ -14044,7 +14044,7 @@
         <v>370</v>
       </c>
       <c r="P96" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q96" s="13" t="s">
         <v>371</v>
@@ -15804,7 +15804,7 @@
       <c r="N134" s="14"/>
       <c r="O134" s="15"/>
       <c r="P134" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q134" s="13" t="s">
         <v>501</v>
@@ -15900,7 +15900,7 @@
         <v>508</v>
       </c>
       <c r="P136" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q136" s="13" t="s">
         <v>509</v>
@@ -15990,7 +15990,7 @@
       <c r="N138" s="14"/>
       <c r="O138" s="15"/>
       <c r="P138" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q138" s="13" t="s">
         <v>514</v>
@@ -16084,7 +16084,7 @@
       </c>
       <c r="O140" s="15"/>
       <c r="P140" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q140" s="13" t="s">
         <v>522</v>
@@ -16986,7 +16986,7 @@
       <c r="N159" s="11"/>
       <c r="O159" s="12"/>
       <c r="P159" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q159" s="13" t="s">
         <v>593</v>
@@ -17508,7 +17508,7 @@
         <v>629</v>
       </c>
       <c r="P170" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q170" s="13" t="s">
         <v>630</v>
@@ -17554,7 +17554,7 @@
       </c>
       <c r="O171" s="12"/>
       <c r="P171" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q171" s="13" t="s">
         <v>634</v>
@@ -18152,7 +18152,7 @@
       <c r="N184" s="11"/>
       <c r="O184" s="12"/>
       <c r="P184" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q184" s="13" t="s">
         <v>669</v>
@@ -18428,7 +18428,7 @@
       </c>
       <c r="O190" s="12"/>
       <c r="P190" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q190" s="13" t="s">
         <v>687</v>
@@ -18720,7 +18720,7 @@
       <c r="N196" s="14"/>
       <c r="O196" s="15"/>
       <c r="P196" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q196" s="13" t="s">
         <v>707</v>
@@ -18862,7 +18862,7 @@
         <v>715</v>
       </c>
       <c r="P199" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q199" s="13" t="s">
         <v>716</v>
@@ -18910,7 +18910,7 @@
         <v>719</v>
       </c>
       <c r="P200" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q200" s="13" t="s">
         <v>720</v>
@@ -18958,7 +18958,7 @@
         <v>370</v>
       </c>
       <c r="P201" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q201" s="13" t="s">
         <v>722</v>
@@ -19472,7 +19472,7 @@
         <v>752</v>
       </c>
       <c r="P212" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q212" s="13" t="s">
         <v>753</v>
@@ -19520,7 +19520,7 @@
         <v>756</v>
       </c>
       <c r="P213" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q213" s="13" t="s">
         <v>757</v>
@@ -19904,7 +19904,7 @@
         <v>786</v>
       </c>
       <c r="P221" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q221" s="13" t="s">
         <v>787</v>
@@ -20378,7 +20378,7 @@
         <v>815</v>
       </c>
       <c r="P231" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q231" s="13" t="s">
         <v>816</v>
@@ -20426,7 +20426,7 @@
         <v>818</v>
       </c>
       <c r="P232" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q232" s="13" t="s">
         <v>819</v>
@@ -20880,7 +20880,7 @@
         <v>853</v>
       </c>
       <c r="P242" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q242" s="15"/>
       <c r="R242" s="14"/>
@@ -21284,7 +21284,7 @@
       <c r="N251" s="14"/>
       <c r="O251" s="15"/>
       <c r="P251" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q251" s="13" t="s">
         <v>875</v>
@@ -21916,7 +21916,7 @@
         <v>922</v>
       </c>
       <c r="P264" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q264" s="13" t="s">
         <v>923</v>
@@ -22008,7 +22008,7 @@
         <v>370</v>
       </c>
       <c r="P266" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q266" s="13" t="s">
         <v>928</v>
@@ -22056,7 +22056,7 @@
         <v>931</v>
       </c>
       <c r="P267" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q267" s="13" t="s">
         <v>932</v>
@@ -22426,7 +22426,7 @@
         <v>949</v>
       </c>
       <c r="P275" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q275" s="13" t="s">
         <v>950</v>
@@ -23018,7 +23018,7 @@
       <c r="N288" s="11"/>
       <c r="O288" s="12"/>
       <c r="P288" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q288" s="13" t="s">
         <v>997</v>
@@ -23064,7 +23064,7 @@
       <c r="N289" s="11"/>
       <c r="O289" s="12"/>
       <c r="P289" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q289" s="13" t="s">
         <v>999</v>
@@ -24482,7 +24482,7 @@
       </c>
       <c r="O319" s="12"/>
       <c r="P319" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q319" s="13" t="s">
         <v>1087</v>
@@ -24880,7 +24880,7 @@
       <c r="N328" s="11"/>
       <c r="O328" s="12"/>
       <c r="P328" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q328" s="13" t="s">
         <v>1110</v>
@@ -25108,7 +25108,7 @@
       <c r="N333" s="11"/>
       <c r="O333" s="12"/>
       <c r="P333" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q333" s="13" t="s">
         <v>1126</v>
@@ -25244,7 +25244,7 @@
       <c r="N336" s="11"/>
       <c r="O336" s="12"/>
       <c r="P336" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q336" s="13" t="s">
         <v>1135</v>
@@ -25380,7 +25380,7 @@
       <c r="N339" s="11"/>
       <c r="O339" s="12"/>
       <c r="P339" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q339" s="13" t="s">
         <v>1145</v>
@@ -25516,7 +25516,7 @@
       <c r="N342" s="11"/>
       <c r="O342" s="12"/>
       <c r="P342" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q342" s="13" t="s">
         <v>1153</v>
@@ -25562,7 +25562,7 @@
       <c r="N343" s="11"/>
       <c r="O343" s="12"/>
       <c r="P343" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q343" s="13" t="s">
         <v>1156</v>
@@ -25718,7 +25718,7 @@
       <c r="N346" s="14"/>
       <c r="O346" s="15"/>
       <c r="P346" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q346" s="13" t="s">
         <v>1166</v>
@@ -25770,7 +25770,7 @@
       <c r="N347" s="14"/>
       <c r="O347" s="15"/>
       <c r="P347" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q347" s="13" t="s">
         <v>1166</v>
@@ -26062,7 +26062,7 @@
         <v>1184</v>
       </c>
       <c r="P353" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q353" s="13" t="s">
         <v>1185</v>
@@ -26626,7 +26626,7 @@
       <c r="N365" s="14"/>
       <c r="O365" s="15"/>
       <c r="P365" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q365" s="13" t="s">
         <v>1213</v>
@@ -26720,7 +26720,7 @@
       <c r="N367" s="14"/>
       <c r="O367" s="15"/>
       <c r="P367" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q367" s="13" t="s">
         <v>1219</v>
@@ -26768,7 +26768,7 @@
       <c r="N368" s="14"/>
       <c r="O368" s="15"/>
       <c r="P368" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q368" s="13" t="s">
         <v>1222</v>
@@ -26816,7 +26816,7 @@
       <c r="N369" s="14"/>
       <c r="O369" s="15"/>
       <c r="P369" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q369" s="13" t="s">
         <v>1224</v>
@@ -26864,7 +26864,7 @@
       <c r="N370" s="14"/>
       <c r="O370" s="15"/>
       <c r="P370" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q370" s="13" t="s">
         <v>1227</v>
@@ -26912,7 +26912,7 @@
       <c r="N371" s="14"/>
       <c r="O371" s="15"/>
       <c r="P371" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q371" s="13" t="s">
         <v>1229</v>
@@ -27200,7 +27200,7 @@
       <c r="N377" s="14"/>
       <c r="O377" s="15"/>
       <c r="P377" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q377" s="13" t="s">
         <v>1246</v>
@@ -27346,7 +27346,7 @@
         <v>1256</v>
       </c>
       <c r="P380" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q380" s="13" t="s">
         <v>1257</v>
@@ -27398,7 +27398,7 @@
         <v>1256</v>
       </c>
       <c r="P381" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q381" s="13" t="s">
         <v>1257</v>
@@ -27588,7 +27588,7 @@
       <c r="N385" s="14"/>
       <c r="O385" s="15"/>
       <c r="P385" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q385" s="13" t="s">
         <v>1271</v>
@@ -27820,7 +27820,7 @@
       <c r="N390" s="14"/>
       <c r="O390" s="15"/>
       <c r="P390" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q390" s="13" t="s">
         <v>1285</v>
@@ -28256,7 +28256,7 @@
       <c r="N399" s="14"/>
       <c r="O399" s="15"/>
       <c r="P399" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q399" s="13" t="s">
         <v>1318</v>
@@ -28306,7 +28306,7 @@
       <c r="N400" s="14"/>
       <c r="O400" s="15"/>
       <c r="P400" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q400" s="13" t="s">
         <v>1322</v>
@@ -28596,7 +28596,7 @@
         <v>472</v>
       </c>
       <c r="P406" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q406" s="13" t="s">
         <v>1339</v>
@@ -28968,7 +28968,7 @@
       </c>
       <c r="O414" s="15"/>
       <c r="P414" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q414" s="13" t="s">
         <v>1358</v>
@@ -29108,7 +29108,7 @@
         <v>1368</v>
       </c>
       <c r="P417" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q417" s="13" t="s">
         <v>1369</v>
@@ -29756,7 +29756,7 @@
         <v>1408</v>
       </c>
       <c r="P430" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q430" s="13" t="s">
         <v>1409</v>
@@ -29800,7 +29800,7 @@
       <c r="N431" s="11"/>
       <c r="O431" s="12"/>
       <c r="P431" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q431" s="13" t="s">
         <v>1412</v>
@@ -29848,7 +29848,7 @@
         <v>472</v>
       </c>
       <c r="P432" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q432" s="13" t="s">
         <v>1414</v>
@@ -29896,7 +29896,7 @@
         <v>1416</v>
       </c>
       <c r="P433" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q433" s="13" t="s">
         <v>1417</v>
@@ -30232,7 +30232,7 @@
       <c r="N440" s="11"/>
       <c r="O440" s="12"/>
       <c r="P440" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q440" s="13" t="s">
         <v>1433</v>
@@ -30280,7 +30280,7 @@
       <c r="N441" s="11"/>
       <c r="O441" s="12"/>
       <c r="P441" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q441" s="13" t="s">
         <v>1436</v>
@@ -30374,7 +30374,7 @@
         <v>1442</v>
       </c>
       <c r="P443" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q443" s="13" t="s">
         <v>1443</v>
@@ -30422,7 +30422,7 @@
         <v>1445</v>
       </c>
       <c r="P444" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q444" s="13" t="s">
         <v>1446</v>
@@ -30472,7 +30472,7 @@
         <v>1448</v>
       </c>
       <c r="P445" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q445" s="13" t="s">
         <v>1449</v>
@@ -30522,7 +30522,7 @@
         <v>1452</v>
       </c>
       <c r="P446" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q446" s="13" t="s">
         <v>1453</v>
@@ -30708,7 +30708,7 @@
       <c r="N450" s="11"/>
       <c r="O450" s="12"/>
       <c r="P450" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q450" s="13" t="s">
         <v>1468</v>
@@ -30752,7 +30752,7 @@
       <c r="N451" s="11"/>
       <c r="O451" s="12"/>
       <c r="P451" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q451" s="13" t="s">
         <v>1471</v>
@@ -30796,7 +30796,7 @@
       <c r="N452" s="11"/>
       <c r="O452" s="12"/>
       <c r="P452" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q452" s="13" t="s">
         <v>1474</v>
@@ -30840,7 +30840,7 @@
       <c r="N453" s="11"/>
       <c r="O453" s="12"/>
       <c r="P453" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q453" s="13" t="s">
         <v>1471</v>
@@ -30980,7 +30980,7 @@
       <c r="N456" s="11"/>
       <c r="O456" s="12"/>
       <c r="P456" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q456" s="13" t="s">
         <v>1486</v>
@@ -31024,7 +31024,7 @@
       <c r="N457" s="11"/>
       <c r="O457" s="12"/>
       <c r="P457" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q457" s="13" t="s">
         <v>1490</v>
@@ -31256,7 +31256,7 @@
         <v>1501</v>
       </c>
       <c r="P462" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q462" s="13" t="s">
         <v>1502</v>
@@ -32350,7 +32350,7 @@
         <v>1561</v>
       </c>
       <c r="P485" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q485" s="13" t="s">
         <v>1562</v>
@@ -32442,7 +32442,7 @@
       <c r="N487" s="11"/>
       <c r="O487" s="12"/>
       <c r="P487" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q487" s="13" t="s">
         <v>1568</v>
@@ -32676,7 +32676,7 @@
         <v>1583</v>
       </c>
       <c r="P492" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q492" s="13" t="s">
         <v>1584</v>
@@ -33122,7 +33122,7 @@
       <c r="N501" s="14"/>
       <c r="O501" s="15"/>
       <c r="P501" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q501" s="13" t="s">
         <v>1610</v>
@@ -33400,7 +33400,7 @@
       <c r="N507" s="14"/>
       <c r="O507" s="15"/>
       <c r="P507" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q507" s="13" t="s">
         <v>1631</v>
@@ -33842,7 +33842,7 @@
         <v>1666</v>
       </c>
       <c r="P516" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q516" s="13" t="s">
         <v>1667</v>
@@ -34202,7 +34202,7 @@
       <c r="N524" s="14"/>
       <c r="O524" s="15"/>
       <c r="P524" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q524" s="13" t="s">
         <v>1690</v>
@@ -34388,7 +34388,7 @@
       <c r="N528" s="14"/>
       <c r="O528" s="15"/>
       <c r="P528" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q528" s="13" t="s">
         <v>1703</v>
@@ -34610,7 +34610,7 @@
       <c r="N533" s="14"/>
       <c r="O533" s="15"/>
       <c r="P533" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q533" s="13" t="s">
         <v>1716</v>
@@ -34750,7 +34750,7 @@
         <v>1726</v>
       </c>
       <c r="P536" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q536" s="13" t="s">
         <v>1727</v>
@@ -35096,7 +35096,7 @@
       <c r="N543" s="14"/>
       <c r="O543" s="15"/>
       <c r="P543" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q543" s="13" t="s">
         <v>1752</v>
@@ -35144,7 +35144,7 @@
         <v>1754</v>
       </c>
       <c r="P544" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q544" s="13" t="s">
         <v>1755</v>
@@ -35192,7 +35192,7 @@
         <v>1758</v>
       </c>
       <c r="P545" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q545" s="13" t="s">
         <v>1759</v>
@@ -35332,7 +35332,7 @@
         <v>1768</v>
       </c>
       <c r="P548" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q548" s="13" t="s">
         <v>1769</v>
@@ -35710,7 +35710,7 @@
         <v>1788</v>
       </c>
       <c r="P556" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q556" s="13" t="s">
         <v>1789</v>
@@ -35850,7 +35850,7 @@
         <v>1798</v>
       </c>
       <c r="P559" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q559" s="13" t="s">
         <v>1799</v>
@@ -35898,7 +35898,7 @@
         <v>1801</v>
       </c>
       <c r="P560" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q560" s="13" t="s">
         <v>1802</v>
@@ -35946,7 +35946,7 @@
         <v>1804</v>
       </c>
       <c r="P561" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q561" s="13" t="s">
         <v>1805</v>
@@ -35992,7 +35992,7 @@
       <c r="N562" s="14"/>
       <c r="O562" s="15"/>
       <c r="P562" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q562" s="13" t="s">
         <v>1809</v>
@@ -36040,7 +36040,7 @@
         <v>1811</v>
       </c>
       <c r="P563" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q563" s="13" t="s">
         <v>1812</v>
@@ -36088,7 +36088,7 @@
         <v>1814</v>
       </c>
       <c r="P564" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q564" s="13" t="s">
         <v>1815</v>
@@ -36134,7 +36134,7 @@
       <c r="N565" s="14"/>
       <c r="O565" s="15"/>
       <c r="P565" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q565" s="13" t="s">
         <v>1817</v>
@@ -36182,7 +36182,7 @@
         <v>1820</v>
       </c>
       <c r="P566" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q566" s="13" t="s">
         <v>1821</v>
@@ -36230,7 +36230,7 @@
         <v>1823</v>
       </c>
       <c r="P567" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q567" s="13" t="s">
         <v>1824</v>
@@ -36278,7 +36278,7 @@
         <v>1827</v>
       </c>
       <c r="P568" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q568" s="13" t="s">
         <v>1828</v>
@@ -36596,7 +36596,7 @@
       <c r="N575" s="14"/>
       <c r="O575" s="15"/>
       <c r="P575" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q575" s="13" t="s">
         <v>1849</v>
@@ -36734,7 +36734,7 @@
       <c r="N578" s="14"/>
       <c r="O578" s="15"/>
       <c r="P578" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q578" s="13" t="s">
         <v>1857</v>
@@ -36778,7 +36778,7 @@
       <c r="N579" s="14"/>
       <c r="O579" s="15"/>
       <c r="P579" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q579" s="13" t="s">
         <v>1859</v>
@@ -36868,7 +36868,7 @@
       </c>
       <c r="O581" s="15"/>
       <c r="P581" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q581" s="13" t="s">
         <v>1865</v>
@@ -37136,7 +37136,7 @@
       <c r="N587" s="14"/>
       <c r="O587" s="15"/>
       <c r="P587" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q587" s="13" t="s">
         <v>1882</v>
@@ -37276,7 +37276,7 @@
         <v>1892</v>
       </c>
       <c r="P590" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q590" s="13" t="s">
         <v>1893</v>
@@ -37966,7 +37966,7 @@
       <c r="N605" s="14"/>
       <c r="O605" s="15"/>
       <c r="P605" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q605" s="13" t="s">
         <v>1938</v>
@@ -39220,7 +39220,7 @@
       <c r="N631" s="11"/>
       <c r="O631" s="12"/>
       <c r="P631" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q631" s="13" t="s">
         <v>2010</v>
@@ -39370,7 +39370,7 @@
       <c r="N634" s="11"/>
       <c r="O634" s="12"/>
       <c r="P634" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q634" s="13" t="s">
         <v>2021</v>
@@ -41174,7 +41174,7 @@
         <v>2150</v>
       </c>
       <c r="P671" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q671" s="13" t="s">
         <v>2151</v>
@@ -41222,7 +41222,7 @@
         <v>472</v>
       </c>
       <c r="P672" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q672" s="13" t="s">
         <v>2153</v>
@@ -41268,7 +41268,7 @@
       <c r="N673" s="14"/>
       <c r="O673" s="15"/>
       <c r="P673" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q673" s="13" t="s">
         <v>2156</v>
@@ -42416,7 +42416,7 @@
       <c r="N697" s="14"/>
       <c r="O697" s="15"/>
       <c r="P697" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q697" s="13" t="s">
         <v>2233</v>
@@ -42710,7 +42710,7 @@
         <v>2254</v>
       </c>
       <c r="P703" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q703" s="13" t="s">
         <v>2255</v>
@@ -43272,7 +43272,7 @@
       <c r="N715" s="14"/>
       <c r="O715" s="15"/>
       <c r="P715" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q715" s="13" t="s">
         <v>2288</v>
@@ -57072,7 +57072,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4BECCB29-AF9D-4FD4-9F87-F72926CA683E}</x14:id>
+          <x14:id>{5350C55E-20C0-47DE-83F6-19478CD1E8D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -57086,7 +57086,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2DE46FF5-C124-4711-B5E2-23AE49739363}</x14:id>
+          <x14:id>{D65F30A8-6071-41E4-B4D1-91162B3870E0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -57100,7 +57100,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{16C97F9A-A868-4DAC-A2B0-15BD208C37C8}</x14:id>
+          <x14:id>{B2636ED8-AE00-4018-A0DF-34DAFD4CF8E0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -57114,7 +57114,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{31905799-8C51-4264-AAF0-F8D9FCC6CF28}</x14:id>
+          <x14:id>{2DA67D50-3049-452B-826D-FBD016D5297C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -57128,7 +57128,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E1824C55-AC2F-406B-9EAE-8678CCCCEACB}</x14:id>
+          <x14:id>{676EBF45-32CD-473E-91D8-2E82A3B9A553}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -57145,7 +57145,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4BECCB29-AF9D-4FD4-9F87-F72926CA683E}">
+          <x14:cfRule type="dataBar" id="{5350C55E-20C0-47DE-83F6-19478CD1E8D0}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -57158,7 +57158,7 @@
           <xm:sqref>B5:B14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2DE46FF5-C124-4711-B5E2-23AE49739363}">
+          <x14:cfRule type="dataBar" id="{D65F30A8-6071-41E4-B4D1-91162B3870E0}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -57171,7 +57171,7 @@
           <xm:sqref>C5:C14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{16C97F9A-A868-4DAC-A2B0-15BD208C37C8}">
+          <x14:cfRule type="dataBar" id="{B2636ED8-AE00-4018-A0DF-34DAFD4CF8E0}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -57184,7 +57184,7 @@
           <xm:sqref>E5:E14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{31905799-8C51-4264-AAF0-F8D9FCC6CF28}">
+          <x14:cfRule type="dataBar" id="{2DA67D50-3049-452B-826D-FBD016D5297C}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -57197,7 +57197,7 @@
           <xm:sqref>F5:F14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E1824C55-AC2F-406B-9EAE-8678CCCCEACB}">
+          <x14:cfRule type="dataBar" id="{676EBF45-32CD-473E-91D8-2E82A3B9A553}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -57301,7 +57301,7 @@
       </c>
       <c r="D11" s="9" t="n">
         <f aca="false">SUMIFS('All weeks'!$L$9:$L$721,'All weeks'!$J$9:$J$721,"A4 90 gsm (booklet)")</f>
-        <v>196</v>
+        <v>364</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>